<commit_message>
added course-sections conflict constraint
- added UI elements necessary to input the conflict information
- tested with set of 2 courses 2 sections : giving feasible solution
- if we add 3+ sections or 3+ courses, it is giving infeasible solution even with soft constraint
- updated import-export functions to adapt to new constraint

Possible TODOs:
- add conflict verification
- add conflict constraint in soft constraints
</commit_message>
<xml_diff>
--- a/static/Timetable_Config_LP.xlsx
+++ b/static/Timetable_Config_LP.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,6 +13,7 @@
     <sheet name="Courses" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Faculty" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Mapping" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Conflicts" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="114">
   <si>
     <t xml:space="preserve">Class Timetable Scheduler Configuration</t>
   </si>
@@ -345,6 +346,27 @@
   </si>
   <si>
     <t xml:space="preserve">Faculty Short Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Courses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EPGP-203, EPGP-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A, B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EPGP-201, EPGP-205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D, E</t>
   </si>
 </sst>
 </file>
@@ -1987,4 +2009,60 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.02"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>